<commit_message>
comment cleanup and added back the 2021 draws missing from the excel
</commit_message>
<xml_diff>
--- a/excel_lotto_records/daily3.xlsx
+++ b/excel_lotto_records/daily3.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,21 +413,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C951"/>
+  <dimension ref="A1:C961"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Unnamed: 0</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Numbers</t>
         </is>
@@ -14692,6 +14680,156 @@
       <c r="C951" t="inlineStr">
         <is>
           <t>9-7-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="952">
+      <c r="A952" t="n">
+        <v>950</v>
+      </c>
+      <c r="B952" t="inlineStr">
+        <is>
+          <t>10/12/2026</t>
+        </is>
+      </c>
+      <c r="C952" t="inlineStr">
+        <is>
+          <t>6-2-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="953">
+      <c r="A953" t="n">
+        <v>951</v>
+      </c>
+      <c r="B953" t="inlineStr">
+        <is>
+          <t>10/13/2026</t>
+        </is>
+      </c>
+      <c r="C953" t="inlineStr">
+        <is>
+          <t>8-0-8</t>
+        </is>
+      </c>
+    </row>
+    <row r="954">
+      <c r="A954" t="n">
+        <v>952</v>
+      </c>
+      <c r="B954" t="inlineStr">
+        <is>
+          <t>10/14/2026</t>
+        </is>
+      </c>
+      <c r="C954" t="inlineStr">
+        <is>
+          <t>8-5-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="955">
+      <c r="A955" t="n">
+        <v>953</v>
+      </c>
+      <c r="B955" t="inlineStr">
+        <is>
+          <t>10/15/2026</t>
+        </is>
+      </c>
+      <c r="C955" t="inlineStr">
+        <is>
+          <t>3-0-7</t>
+        </is>
+      </c>
+    </row>
+    <row r="956">
+      <c r="A956" t="n">
+        <v>954</v>
+      </c>
+      <c r="B956" t="inlineStr">
+        <is>
+          <t>10/16/2026</t>
+        </is>
+      </c>
+      <c r="C956" t="inlineStr">
+        <is>
+          <t>7-1-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="957">
+      <c r="A957" t="n">
+        <v>955</v>
+      </c>
+      <c r="B957" t="inlineStr">
+        <is>
+          <t>10/17/2026</t>
+        </is>
+      </c>
+      <c r="C957" t="inlineStr">
+        <is>
+          <t>4-4-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="958">
+      <c r="A958" t="n">
+        <v>956</v>
+      </c>
+      <c r="B958" t="inlineStr">
+        <is>
+          <t>10/19/2026</t>
+        </is>
+      </c>
+      <c r="C958" t="inlineStr">
+        <is>
+          <t>2-9-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="959">
+      <c r="A959" t="n">
+        <v>957</v>
+      </c>
+      <c r="B959" t="inlineStr">
+        <is>
+          <t>10/20/2026</t>
+        </is>
+      </c>
+      <c r="C959" t="inlineStr">
+        <is>
+          <t>5-7-6</t>
+        </is>
+      </c>
+    </row>
+    <row r="960">
+      <c r="A960" t="n">
+        <v>958</v>
+      </c>
+      <c r="B960" t="inlineStr">
+        <is>
+          <t>10/21/2026</t>
+        </is>
+      </c>
+      <c r="C960" t="inlineStr">
+        <is>
+          <t>1-6-6</t>
+        </is>
+      </c>
+    </row>
+    <row r="961">
+      <c r="A961" t="n">
+        <v>959</v>
+      </c>
+      <c r="B961" t="inlineStr">
+        <is>
+          <t>10/22/2026</t>
+        </is>
+      </c>
+      <c r="C961" t="inlineStr">
+        <is>
+          <t>2-5-1</t>
         </is>
       </c>
     </row>

</xml_diff>